<commit_message>
Restore KTAM name so real Source files match
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TWYDySAGURhagPjRB9vvPw
</commit_message>
<xml_diff>
--- a/sample-data/ข้อมูลสมมติ_AUM_NetFlow.xlsx
+++ b/sample-data/ข้อมูลสมมติ_AUM_NetFlow.xlsx
@@ -629,7 +629,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -719,7 +719,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F151" t="n">
@@ -7649,7 +7649,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -8189,7 +8189,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -9809,7 +9809,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F208" t="n">
@@ -10304,7 +10304,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F219" t="n">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F239" t="n">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F244" t="n">
@@ -11699,7 +11699,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F250" t="n">
@@ -11789,7 +11789,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F252" t="n">
@@ -12149,7 +12149,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F260" t="n">
@@ -12509,7 +12509,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -13184,7 +13184,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -13454,7 +13454,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F289" t="n">
@@ -14264,7 +14264,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F307" t="n">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -14849,7 +14849,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F320" t="n">
@@ -14894,7 +14894,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F321" t="n">
@@ -15659,7 +15659,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F338" t="n">
@@ -16109,7 +16109,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F348" t="n">
@@ -16154,7 +16154,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F349" t="n">
@@ -16694,7 +16694,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F361" t="n">
@@ -17144,7 +17144,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F371" t="n">
@@ -17369,7 +17369,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F376" t="n">
@@ -17729,7 +17729,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F384" t="n">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F389" t="n">
@@ -17999,7 +17999,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F390" t="n">
@@ -18089,7 +18089,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F392" t="n">
@@ -20159,7 +20159,7 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F438" t="n">
@@ -20249,7 +20249,7 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F440" t="n">
@@ -20744,7 +20744,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F451" t="n">
@@ -20924,7 +20924,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F455" t="n">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F457" t="n">
@@ -21104,7 +21104,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F459" t="n">
@@ -21374,7 +21374,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F465" t="n">
@@ -21509,7 +21509,7 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F468" t="n">
@@ -21824,7 +21824,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F475" t="n">
@@ -21914,7 +21914,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F477" t="n">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F480" t="n">
@@ -22094,7 +22094,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F481" t="n">
@@ -23354,7 +23354,7 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F509" t="n">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="E536" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F536" t="n">
@@ -24659,7 +24659,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F538" t="n">
@@ -25154,7 +25154,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F549" t="n">
@@ -26144,7 +26144,7 @@
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F571" t="n">
@@ -26279,7 +26279,7 @@
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F574" t="n">
@@ -26684,7 +26684,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F583" t="n">
@@ -26819,7 +26819,7 @@
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F586" t="n">
@@ -27179,7 +27179,7 @@
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F594" t="n">
@@ -27314,7 +27314,7 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F597" t="n">
@@ -27359,7 +27359,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F598" t="n">
@@ -27854,7 +27854,7 @@
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F609" t="n">
@@ -27944,7 +27944,7 @@
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F611" t="n">
@@ -28889,7 +28889,7 @@
       </c>
       <c r="E632" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F632" t="n">
@@ -29249,7 +29249,7 @@
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F640" t="n">
@@ -29339,7 +29339,7 @@
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F642" t="n">
@@ -29564,7 +29564,7 @@
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F647" t="n">
@@ -29609,7 +29609,7 @@
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F648" t="n">
@@ -29879,7 +29879,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F654" t="n">
@@ -30509,7 +30509,7 @@
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F668" t="n">
@@ -30644,7 +30644,7 @@
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F671" t="n">
@@ -30824,7 +30824,7 @@
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F675" t="n">
@@ -31499,7 +31499,7 @@
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F690" t="n">
@@ -31679,7 +31679,7 @@
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F694" t="n">
@@ -31769,7 +31769,7 @@
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F696" t="n">
@@ -33029,7 +33029,7 @@
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F724" t="n">
@@ -33119,7 +33119,7 @@
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F726" t="n">
@@ -33254,7 +33254,7 @@
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F729" t="n">
@@ -33389,7 +33389,7 @@
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F732" t="n">
@@ -33794,7 +33794,7 @@
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F741" t="n">
@@ -34334,7 +34334,7 @@
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F753" t="n">
@@ -34379,7 +34379,7 @@
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F754" t="n">
@@ -34469,7 +34469,7 @@
       </c>
       <c r="E756" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F756" t="n">
@@ -34739,7 +34739,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F762" t="n">
@@ -34784,7 +34784,7 @@
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F763" t="n">
@@ -35054,7 +35054,7 @@
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F769" t="n">
@@ -35279,7 +35279,7 @@
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F774" t="n">
@@ -35549,7 +35549,7 @@
       </c>
       <c r="E780" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F780" t="n">
@@ -35909,7 +35909,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F788" t="n">
@@ -36854,7 +36854,7 @@
       </c>
       <c r="E809" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F809" t="n">
@@ -36944,7 +36944,7 @@
       </c>
       <c r="E811" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F811" t="n">
@@ -37664,7 +37664,7 @@
       </c>
       <c r="E827" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F827" t="n">
@@ -37709,7 +37709,7 @@
       </c>
       <c r="E828" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F828" t="n">
@@ -38159,7 +38159,7 @@
       </c>
       <c r="E838" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F838" t="n">
@@ -38294,7 +38294,7 @@
       </c>
       <c r="E841" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F841" t="n">
@@ -38699,7 +38699,7 @@
       </c>
       <c r="E850" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F850" t="n">
@@ -39014,7 +39014,7 @@
       </c>
       <c r="E857" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F857" t="n">
@@ -39149,7 +39149,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F860" t="n">
@@ -39239,7 +39239,7 @@
       </c>
       <c r="E862" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F862" t="n">
@@ -39419,7 +39419,7 @@
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F866" t="n">
@@ -40184,7 +40184,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F883" t="n">
@@ -40859,7 +40859,7 @@
       </c>
       <c r="E898" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F898" t="n">
@@ -41354,7 +41354,7 @@
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F909" t="n">
@@ -41939,7 +41939,7 @@
       </c>
       <c r="E922" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F922" t="n">
@@ -42164,7 +42164,7 @@
       </c>
       <c r="E927" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F927" t="n">
@@ -42254,7 +42254,7 @@
       </c>
       <c r="E929" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F929" t="n">
@@ -42479,7 +42479,7 @@
       </c>
       <c r="E934" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F934" t="n">
@@ -42749,7 +42749,7 @@
       </c>
       <c r="E940" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F940" t="n">
@@ -42839,7 +42839,7 @@
       </c>
       <c r="E942" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F942" t="n">
@@ -43199,7 +43199,7 @@
       </c>
       <c r="E950" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F950" t="n">
@@ -43559,7 +43559,7 @@
       </c>
       <c r="E958" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F958" t="n">
@@ -44234,7 +44234,7 @@
       </c>
       <c r="E973" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F973" t="n">
@@ -44504,7 +44504,7 @@
       </c>
       <c r="E979" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F979" t="n">
@@ -45314,7 +45314,7 @@
       </c>
       <c r="E997" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F997" t="n">
@@ -45584,7 +45584,7 @@
       </c>
       <c r="E1003" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1003" t="n">
@@ -45899,7 +45899,7 @@
       </c>
       <c r="E1010" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1010" t="n">
@@ -45944,7 +45944,7 @@
       </c>
       <c r="E1011" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1011" t="n">
@@ -46709,7 +46709,7 @@
       </c>
       <c r="E1028" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1028" t="n">
@@ -47159,7 +47159,7 @@
       </c>
       <c r="E1038" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1038" t="n">
@@ -47204,7 +47204,7 @@
       </c>
       <c r="E1039" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1039" t="n">
@@ -47744,7 +47744,7 @@
       </c>
       <c r="E1051" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1051" t="n">
@@ -48194,7 +48194,7 @@
       </c>
       <c r="E1061" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1061" t="n">
@@ -48419,7 +48419,7 @@
       </c>
       <c r="E1066" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1066" t="n">
@@ -48779,7 +48779,7 @@
       </c>
       <c r="E1074" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1074" t="n">
@@ -49004,7 +49004,7 @@
       </c>
       <c r="E1079" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1079" t="n">
@@ -49049,7 +49049,7 @@
       </c>
       <c r="E1080" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1080" t="n">
@@ -49139,7 +49139,7 @@
       </c>
       <c r="E1082" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1082" t="n">
@@ -51209,7 +51209,7 @@
       </c>
       <c r="E1128" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1128" t="n">
@@ -51299,7 +51299,7 @@
       </c>
       <c r="E1130" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1130" t="n">
@@ -51794,7 +51794,7 @@
       </c>
       <c r="E1141" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1141" t="n">
@@ -51974,7 +51974,7 @@
       </c>
       <c r="E1145" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1145" t="n">
@@ -52064,7 +52064,7 @@
       </c>
       <c r="E1147" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1147" t="n">
@@ -52154,7 +52154,7 @@
       </c>
       <c r="E1149" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1149" t="n">
@@ -52424,7 +52424,7 @@
       </c>
       <c r="E1155" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1155" t="n">
@@ -52559,7 +52559,7 @@
       </c>
       <c r="E1158" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1158" t="n">
@@ -52874,7 +52874,7 @@
       </c>
       <c r="E1165" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1165" t="n">
@@ -52964,7 +52964,7 @@
       </c>
       <c r="E1167" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1167" t="n">
@@ -53099,7 +53099,7 @@
       </c>
       <c r="E1170" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1170" t="n">
@@ -53144,7 +53144,7 @@
       </c>
       <c r="E1171" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1171" t="n">
@@ -54404,7 +54404,7 @@
       </c>
       <c r="E1199" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1199" t="n">
@@ -55619,7 +55619,7 @@
       </c>
       <c r="E1226" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1226" t="n">
@@ -55709,7 +55709,7 @@
       </c>
       <c r="E1228" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1228" t="n">
@@ -56204,7 +56204,7 @@
       </c>
       <c r="E1239" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1239" t="n">
@@ -57194,7 +57194,7 @@
       </c>
       <c r="E1261" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1261" t="n">
@@ -57329,7 +57329,7 @@
       </c>
       <c r="E1264" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1264" t="n">
@@ -57734,7 +57734,7 @@
       </c>
       <c r="E1273" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1273" t="n">
@@ -57869,7 +57869,7 @@
       </c>
       <c r="E1276" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1276" t="n">
@@ -58229,7 +58229,7 @@
       </c>
       <c r="E1284" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1284" t="n">
@@ -58364,7 +58364,7 @@
       </c>
       <c r="E1287" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1287" t="n">
@@ -58409,7 +58409,7 @@
       </c>
       <c r="E1288" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1288" t="n">
@@ -58904,7 +58904,7 @@
       </c>
       <c r="E1299" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1299" t="n">
@@ -58994,7 +58994,7 @@
       </c>
       <c r="E1301" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1301" t="n">
@@ -59939,7 +59939,7 @@
       </c>
       <c r="E1322" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1322" t="n">
@@ -60299,7 +60299,7 @@
       </c>
       <c r="E1330" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1330" t="n">
@@ -60389,7 +60389,7 @@
       </c>
       <c r="E1332" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1332" t="n">
@@ -60614,7 +60614,7 @@
       </c>
       <c r="E1337" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1337" t="n">
@@ -60659,7 +60659,7 @@
       </c>
       <c r="E1338" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1338" t="n">
@@ -60929,7 +60929,7 @@
       </c>
       <c r="E1344" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1344" t="n">
@@ -61559,7 +61559,7 @@
       </c>
       <c r="E1358" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1358" t="n">
@@ -61694,7 +61694,7 @@
       </c>
       <c r="E1361" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1361" t="n">
@@ -61874,7 +61874,7 @@
       </c>
       <c r="E1365" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1365" t="n">
@@ -62549,7 +62549,7 @@
       </c>
       <c r="E1380" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1380" t="n">
@@ -62729,7 +62729,7 @@
       </c>
       <c r="E1384" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1384" t="n">
@@ -62819,7 +62819,7 @@
       </c>
       <c r="E1386" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1386" t="n">
@@ -64079,7 +64079,7 @@
       </c>
       <c r="E1414" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1414" t="n">
@@ -64169,7 +64169,7 @@
       </c>
       <c r="E1416" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1416" t="n">
@@ -64304,7 +64304,7 @@
       </c>
       <c r="E1419" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1419" t="n">
@@ -64439,7 +64439,7 @@
       </c>
       <c r="E1422" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1422" t="n">
@@ -64844,7 +64844,7 @@
       </c>
       <c r="E1431" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1431" t="n">
@@ -65384,7 +65384,7 @@
       </c>
       <c r="E1443" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1443" t="n">
@@ -65429,7 +65429,7 @@
       </c>
       <c r="E1444" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1444" t="n">
@@ -65519,7 +65519,7 @@
       </c>
       <c r="E1446" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1446" t="n">
@@ -65789,7 +65789,7 @@
       </c>
       <c r="E1452" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1452" t="n">
@@ -65834,7 +65834,7 @@
       </c>
       <c r="E1453" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1453" t="n">
@@ -66104,7 +66104,7 @@
       </c>
       <c r="E1459" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1459" t="n">
@@ -66329,7 +66329,7 @@
       </c>
       <c r="E1464" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1464" t="n">
@@ -66599,7 +66599,7 @@
       </c>
       <c r="E1470" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1470" t="n">
@@ -66959,7 +66959,7 @@
       </c>
       <c r="E1478" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1478" t="n">
@@ -67904,7 +67904,7 @@
       </c>
       <c r="E1499" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1499" t="n">
@@ -67994,7 +67994,7 @@
       </c>
       <c r="E1501" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1501" t="n">
@@ -68714,7 +68714,7 @@
       </c>
       <c r="E1517" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1517" t="n">
@@ -68759,7 +68759,7 @@
       </c>
       <c r="E1518" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1518" t="n">
@@ -69209,7 +69209,7 @@
       </c>
       <c r="E1528" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1528" t="n">
@@ -69344,7 +69344,7 @@
       </c>
       <c r="E1531" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1531" t="n">
@@ -69749,7 +69749,7 @@
       </c>
       <c r="E1540" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1540" t="n">
@@ -70064,7 +70064,7 @@
       </c>
       <c r="E1547" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1547" t="n">
@@ -70199,7 +70199,7 @@
       </c>
       <c r="E1550" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1550" t="n">
@@ -70289,7 +70289,7 @@
       </c>
       <c r="E1552" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1552" t="n">
@@ -70469,7 +70469,7 @@
       </c>
       <c r="E1556" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1556" t="n">
@@ -71234,7 +71234,7 @@
       </c>
       <c r="E1573" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1573" t="n">
@@ -71909,7 +71909,7 @@
       </c>
       <c r="E1588" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1588" t="n">
@@ -72404,7 +72404,7 @@
       </c>
       <c r="E1599" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1599" t="n">
@@ -72989,7 +72989,7 @@
       </c>
       <c r="E1612" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1612" t="n">
@@ -73214,7 +73214,7 @@
       </c>
       <c r="E1617" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1617" t="n">
@@ -73304,7 +73304,7 @@
       </c>
       <c r="E1619" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1619" t="n">
@@ -73529,7 +73529,7 @@
       </c>
       <c r="E1624" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1624" t="n">
@@ -73799,7 +73799,7 @@
       </c>
       <c r="E1630" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1630" t="n">
@@ -73889,7 +73889,7 @@
       </c>
       <c r="E1632" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1632" t="n">
@@ -74249,7 +74249,7 @@
       </c>
       <c r="E1640" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1640" t="n">
@@ -74609,7 +74609,7 @@
       </c>
       <c r="E1648" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1648" t="n">
@@ -75284,7 +75284,7 @@
       </c>
       <c r="E1663" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1663" t="n">
@@ -75554,7 +75554,7 @@
       </c>
       <c r="E1669" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1669" t="n">
@@ -76364,7 +76364,7 @@
       </c>
       <c r="E1687" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1687" t="n">
@@ -76634,7 +76634,7 @@
       </c>
       <c r="E1693" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1693" t="n">
@@ -76949,7 +76949,7 @@
       </c>
       <c r="E1700" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1700" t="n">
@@ -76994,7 +76994,7 @@
       </c>
       <c r="E1701" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1701" t="n">
@@ -77759,7 +77759,7 @@
       </c>
       <c r="E1718" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1718" t="n">
@@ -78209,7 +78209,7 @@
       </c>
       <c r="E1728" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1728" t="n">
@@ -78254,7 +78254,7 @@
       </c>
       <c r="E1729" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1729" t="n">
@@ -78794,7 +78794,7 @@
       </c>
       <c r="E1741" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1741" t="n">
@@ -79244,7 +79244,7 @@
       </c>
       <c r="E1751" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1751" t="n">
@@ -79469,7 +79469,7 @@
       </c>
       <c r="E1756" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1756" t="n">
@@ -79829,7 +79829,7 @@
       </c>
       <c r="E1764" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1764" t="n">
@@ -80054,7 +80054,7 @@
       </c>
       <c r="E1769" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1769" t="n">
@@ -80099,7 +80099,7 @@
       </c>
       <c r="E1770" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1770" t="n">
@@ -80189,7 +80189,7 @@
       </c>
       <c r="E1772" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1772" t="n">
@@ -82259,7 +82259,7 @@
       </c>
       <c r="E1818" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1818" t="n">
@@ -82349,7 +82349,7 @@
       </c>
       <c r="E1820" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1820" t="n">
@@ -82844,7 +82844,7 @@
       </c>
       <c r="E1831" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1831" t="n">
@@ -83024,7 +83024,7 @@
       </c>
       <c r="E1835" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1835" t="n">
@@ -83114,7 +83114,7 @@
       </c>
       <c r="E1837" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1837" t="n">
@@ -83204,7 +83204,7 @@
       </c>
       <c r="E1839" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1839" t="n">
@@ -83474,7 +83474,7 @@
       </c>
       <c r="E1845" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1845" t="n">
@@ -83609,7 +83609,7 @@
       </c>
       <c r="E1848" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1848" t="n">
@@ -83924,7 +83924,7 @@
       </c>
       <c r="E1855" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1855" t="n">
@@ -84014,7 +84014,7 @@
       </c>
       <c r="E1857" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1857" t="n">
@@ -84149,7 +84149,7 @@
       </c>
       <c r="E1860" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1860" t="n">
@@ -84194,7 +84194,7 @@
       </c>
       <c r="E1861" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1861" t="n">
@@ -85454,7 +85454,7 @@
       </c>
       <c r="E1889" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1889" t="n">
@@ -86669,7 +86669,7 @@
       </c>
       <c r="E1916" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1916" t="n">
@@ -86759,7 +86759,7 @@
       </c>
       <c r="E1918" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1918" t="n">
@@ -87254,7 +87254,7 @@
       </c>
       <c r="E1929" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1929" t="n">
@@ -88244,7 +88244,7 @@
       </c>
       <c r="E1951" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1951" t="n">
@@ -88379,7 +88379,7 @@
       </c>
       <c r="E1954" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1954" t="n">
@@ -88784,7 +88784,7 @@
       </c>
       <c r="E1963" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1963" t="n">
@@ -88919,7 +88919,7 @@
       </c>
       <c r="E1966" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1966" t="n">
@@ -89279,7 +89279,7 @@
       </c>
       <c r="E1974" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1974" t="n">
@@ -89414,7 +89414,7 @@
       </c>
       <c r="E1977" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1977" t="n">
@@ -89459,7 +89459,7 @@
       </c>
       <c r="E1978" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1978" t="n">
@@ -89954,7 +89954,7 @@
       </c>
       <c r="E1989" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1989" t="n">
@@ -90044,7 +90044,7 @@
       </c>
       <c r="E1991" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F1991" t="n">
@@ -90989,7 +90989,7 @@
       </c>
       <c r="E2012" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2012" t="n">
@@ -91349,7 +91349,7 @@
       </c>
       <c r="E2020" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2020" t="n">
@@ -91439,7 +91439,7 @@
       </c>
       <c r="E2022" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2022" t="n">
@@ -91664,7 +91664,7 @@
       </c>
       <c r="E2027" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2027" t="n">
@@ -91709,7 +91709,7 @@
       </c>
       <c r="E2028" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2028" t="n">
@@ -91979,7 +91979,7 @@
       </c>
       <c r="E2034" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2034" t="n">
@@ -92609,7 +92609,7 @@
       </c>
       <c r="E2048" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2048" t="n">
@@ -92744,7 +92744,7 @@
       </c>
       <c r="E2051" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2051" t="n">
@@ -92924,7 +92924,7 @@
       </c>
       <c r="E2055" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2055" t="n">
@@ -93599,7 +93599,7 @@
       </c>
       <c r="E2070" t="inlineStr">
         <is>
-          <t>Demo Asset Management Co., Ltd.</t>
+          <t>Krungthai Asset Management PLC</t>
         </is>
       </c>
       <c r="F2070" t="n">

</xml_diff>